<commit_message>
Ajout des numéros KABBU dans vto_list
</commit_message>
<xml_diff>
--- a/LOUMAS REPORTING HEBDO PAR VTO _SIMS.xlsx
+++ b/LOUMAS REPORTING HEBDO PAR VTO _SIMS.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView minimized="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil2" sheetId="2" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="SYNT PARTENAIRE LOUMA FEV" sheetId="3" r:id="rId9"/>
     <sheet name="SYNTHESE PARTENAIRE LOUMA MARS" sheetId="9" r:id="rId10"/>
     <sheet name="ND PARTENAIRE" sheetId="10" r:id="rId11"/>
+    <sheet name="Feuil3" sheetId="15" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'SYNT PAIEMENT CHAUF &amp; VTO FEVRI'!$A$1:$V$32</definedName>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="180">
   <si>
     <t>PVT</t>
   </si>
@@ -615,6 +616,36 @@
   <si>
     <t>SEM14</t>
   </si>
+  <si>
+    <t>NORD</t>
+  </si>
+  <si>
+    <t> 776003741</t>
+  </si>
+  <si>
+    <t> 787095631</t>
+  </si>
+  <si>
+    <t> 787095625</t>
+  </si>
+  <si>
+    <t> Pvt_mbpling173</t>
+  </si>
+  <si>
+    <t> 776006374</t>
+  </si>
+  <si>
+    <t>CENTRE</t>
+  </si>
+  <si>
+    <t>OUSMANE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NDIAYE </t>
+  </si>
+  <si>
+    <t>pvt_tcg_0078</t>
+  </si>
 </sst>
 </file>
 
@@ -624,7 +655,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* ###0_-;\-* ###0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -685,8 +716,33 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="18"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -807,8 +863,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1A983"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="31">
+  <borders count="49">
     <border>
       <left/>
       <right/>
@@ -1170,13 +1232,261 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="217">
+  <cellXfs count="241">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1644,6 +1954,21 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1653,45 +1978,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1701,15 +2020,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="12" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1727,6 +2037,78 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="17" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2074,6 +2456,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:solidFill>
@@ -2169,6 +2552,7 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
                 <c15:leaderLines>
                   <c:spPr>
@@ -2351,7 +2735,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:solidFill>
@@ -2447,7 +2830,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
                 <c15:leaderLines>
                   <c:spPr>
@@ -5513,6 +5895,456 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
+  <sheetData>
+    <row r="1" spans="1:6" ht="28" thickBot="1">
+      <c r="A1" s="217"/>
+      <c r="B1" s="218" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="219" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="219" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="219" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="220" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="25.5">
+      <c r="A2" s="235" t="s">
+        <v>139</v>
+      </c>
+      <c r="B2" s="238" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="221" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="221" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="221" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="222">
+        <v>775810336</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="38">
+      <c r="A3" s="236"/>
+      <c r="B3" s="239"/>
+      <c r="C3" s="223" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="223" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="223" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="224">
+        <v>772107591</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="25.5">
+      <c r="A4" s="236"/>
+      <c r="B4" s="239"/>
+      <c r="C4" s="223" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="223" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="223" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="224">
+        <v>772104981</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="26" thickBot="1">
+      <c r="A5" s="237"/>
+      <c r="B5" s="240"/>
+      <c r="C5" s="225" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="225" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="225" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="226">
+        <v>778525987</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="235" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="238" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="221" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="221" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="221" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="227" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="25.5">
+      <c r="A7" s="236"/>
+      <c r="B7" s="239"/>
+      <c r="C7" s="223" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="223" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="223" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="228" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="236"/>
+      <c r="B8" s="239"/>
+      <c r="C8" s="223" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="223" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="223" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" s="228" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="26" thickBot="1">
+      <c r="A9" s="237"/>
+      <c r="B9" s="240"/>
+      <c r="C9" s="225" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="225" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" s="225" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" s="229" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="25.5">
+      <c r="A10" s="235" t="s">
+        <v>140</v>
+      </c>
+      <c r="B10" s="238" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="221" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="221" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="221" t="s">
+        <v>42</v>
+      </c>
+      <c r="F10" s="222" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="25.5">
+      <c r="A11" s="236"/>
+      <c r="B11" s="239"/>
+      <c r="C11" s="223" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="223" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" s="223" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" s="230" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="25.5">
+      <c r="A12" s="236"/>
+      <c r="B12" s="239"/>
+      <c r="C12" s="223" t="s">
+        <v>47</v>
+      </c>
+      <c r="D12" s="223" t="s">
+        <v>48</v>
+      </c>
+      <c r="E12" s="223" t="s">
+        <v>49</v>
+      </c>
+      <c r="F12" s="224">
+        <v>778528509</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="26" thickBot="1">
+      <c r="A13" s="237"/>
+      <c r="B13" s="240"/>
+      <c r="C13" s="225" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" s="225" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="225" t="s">
+        <v>51</v>
+      </c>
+      <c r="F13" s="226">
+        <v>787655222</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="25.5">
+      <c r="A14" s="235" t="s">
+        <v>170</v>
+      </c>
+      <c r="B14" s="238" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="221" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="221" t="s">
+        <v>55</v>
+      </c>
+      <c r="E14" s="221" t="s">
+        <v>56</v>
+      </c>
+      <c r="F14" s="227" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="25.5">
+      <c r="A15" s="236"/>
+      <c r="B15" s="239"/>
+      <c r="C15" s="223" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" s="223" t="s">
+        <v>59</v>
+      </c>
+      <c r="E15" s="223" t="s">
+        <v>60</v>
+      </c>
+      <c r="F15" s="228" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="25.5">
+      <c r="A16" s="236"/>
+      <c r="B16" s="239"/>
+      <c r="C16" s="223" t="s">
+        <v>62</v>
+      </c>
+      <c r="D16" s="223" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" s="223" t="s">
+        <v>63</v>
+      </c>
+      <c r="F16" s="228" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="25.5" thickBot="1">
+      <c r="A17" s="237"/>
+      <c r="B17" s="240"/>
+      <c r="C17" s="231" t="s">
+        <v>65</v>
+      </c>
+      <c r="D17" s="232" t="s">
+        <v>66</v>
+      </c>
+      <c r="E17" s="232" t="s">
+        <v>174</v>
+      </c>
+      <c r="F17" s="233" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="26" thickBot="1">
+      <c r="A18" s="235" t="s">
+        <v>176</v>
+      </c>
+      <c r="B18" s="238" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="221" t="s">
+        <v>70</v>
+      </c>
+      <c r="D18" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="221" t="s">
+        <v>71</v>
+      </c>
+      <c r="F18" s="234">
+        <v>786241255</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="26" thickBot="1">
+      <c r="A19" s="236"/>
+      <c r="B19" s="239"/>
+      <c r="C19" s="223" t="s">
+        <v>72</v>
+      </c>
+      <c r="D19" s="223" t="s">
+        <v>73</v>
+      </c>
+      <c r="E19" s="223" t="s">
+        <v>74</v>
+      </c>
+      <c r="F19" s="234">
+        <v>775812208</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="26" thickBot="1">
+      <c r="A20" s="236"/>
+      <c r="B20" s="239"/>
+      <c r="C20" s="223" t="s">
+        <v>75</v>
+      </c>
+      <c r="D20" s="223" t="s">
+        <v>76</v>
+      </c>
+      <c r="E20" s="223" t="s">
+        <v>77</v>
+      </c>
+      <c r="F20" s="234">
+        <v>786241266</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="26" thickBot="1">
+      <c r="A21" s="237"/>
+      <c r="B21" s="240"/>
+      <c r="C21" s="225" t="s">
+        <v>78</v>
+      </c>
+      <c r="D21" s="225" t="s">
+        <v>79</v>
+      </c>
+      <c r="E21" s="225" t="s">
+        <v>80</v>
+      </c>
+      <c r="F21" s="234">
+        <v>786239376</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="235" t="s">
+        <v>81</v>
+      </c>
+      <c r="B22" s="238" t="s">
+        <v>82</v>
+      </c>
+      <c r="C22" s="221" t="s">
+        <v>83</v>
+      </c>
+      <c r="D22" s="221" t="s">
+        <v>84</v>
+      </c>
+      <c r="E22" s="221" t="s">
+        <v>85</v>
+      </c>
+      <c r="F22" s="227">
+        <v>787095594</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="25.5">
+      <c r="A23" s="236"/>
+      <c r="B23" s="239"/>
+      <c r="C23" s="223" t="s">
+        <v>86</v>
+      </c>
+      <c r="D23" s="223" t="s">
+        <v>87</v>
+      </c>
+      <c r="E23" s="223" t="s">
+        <v>88</v>
+      </c>
+      <c r="F23" s="228">
+        <v>787095584</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="236"/>
+      <c r="B24" s="239"/>
+      <c r="C24" s="223" t="s">
+        <v>89</v>
+      </c>
+      <c r="D24" s="223" t="s">
+        <v>31</v>
+      </c>
+      <c r="E24" s="223" t="s">
+        <v>90</v>
+      </c>
+      <c r="F24" s="228">
+        <v>782989910</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="14.5" thickBot="1">
+      <c r="A25" s="237"/>
+      <c r="B25" s="240"/>
+      <c r="C25" s="225" t="s">
+        <v>177</v>
+      </c>
+      <c r="D25" s="225" t="s">
+        <v>178</v>
+      </c>
+      <c r="E25" s="225" t="s">
+        <v>179</v>
+      </c>
+      <c r="F25" s="229">
+        <v>777411462</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="B10:B13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:Z28"/>
@@ -5603,7 +6435,7 @@
       <c r="B3" s="186" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="196" t="s">
+      <c r="C3" s="189" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="5" t="s">
@@ -5663,7 +6495,7 @@
     </row>
     <row r="4" spans="2:26">
       <c r="B4" s="187"/>
-      <c r="C4" s="196"/>
+      <c r="C4" s="189"/>
       <c r="D4" s="1" t="s">
         <v>12</v>
       </c>
@@ -5721,7 +6553,7 @@
     </row>
     <row r="5" spans="2:26">
       <c r="B5" s="187"/>
-      <c r="C5" s="196"/>
+      <c r="C5" s="189"/>
       <c r="D5" s="1" t="s">
         <v>15</v>
       </c>
@@ -5779,7 +6611,7 @@
     </row>
     <row r="6" spans="2:26" ht="14.5" thickBot="1">
       <c r="B6" s="188"/>
-      <c r="C6" s="197"/>
+      <c r="C6" s="190"/>
       <c r="D6" s="11" t="s">
         <v>15</v>
       </c>
@@ -5839,7 +6671,7 @@
       <c r="B7" s="180" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="192" t="s">
+      <c r="C7" s="191" t="s">
         <v>21</v>
       </c>
       <c r="D7" s="5" t="s">
@@ -5899,7 +6731,7 @@
     </row>
     <row r="8" spans="2:26">
       <c r="B8" s="181"/>
-      <c r="C8" s="193"/>
+      <c r="C8" s="192"/>
       <c r="D8" s="1" t="s">
         <v>26</v>
       </c>
@@ -5957,7 +6789,7 @@
     </row>
     <row r="9" spans="2:26">
       <c r="B9" s="181"/>
-      <c r="C9" s="193"/>
+      <c r="C9" s="192"/>
       <c r="D9" s="1" t="s">
         <v>30</v>
       </c>
@@ -6015,7 +6847,7 @@
     </row>
     <row r="10" spans="2:26" ht="14.5" thickBot="1">
       <c r="B10" s="182"/>
-      <c r="C10" s="198"/>
+      <c r="C10" s="193"/>
       <c r="D10" s="11" t="s">
         <v>34</v>
       </c>
@@ -6075,7 +6907,7 @@
       <c r="B11" s="180" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="192" t="s">
+      <c r="C11" s="191" t="s">
         <v>39</v>
       </c>
       <c r="D11" s="5" t="s">
@@ -6135,7 +6967,7 @@
     </row>
     <row r="12" spans="2:26">
       <c r="B12" s="181"/>
-      <c r="C12" s="193"/>
+      <c r="C12" s="192"/>
       <c r="D12" s="1" t="s">
         <v>22</v>
       </c>
@@ -6193,7 +7025,7 @@
     </row>
     <row r="13" spans="2:26">
       <c r="B13" s="181"/>
-      <c r="C13" s="193"/>
+      <c r="C13" s="192"/>
       <c r="D13" s="1" t="s">
         <v>47</v>
       </c>
@@ -6251,7 +7083,7 @@
     </row>
     <row r="14" spans="2:26" ht="14.5" thickBot="1">
       <c r="B14" s="182"/>
-      <c r="C14" s="198"/>
+      <c r="C14" s="193"/>
       <c r="D14" s="11" t="s">
         <v>50</v>
       </c>
@@ -6311,7 +7143,7 @@
       <c r="B15" s="180" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="189" t="s">
+      <c r="C15" s="194" t="s">
         <v>53</v>
       </c>
       <c r="D15" s="5" t="s">
@@ -6371,7 +7203,7 @@
     </row>
     <row r="16" spans="2:26">
       <c r="B16" s="181"/>
-      <c r="C16" s="190"/>
+      <c r="C16" s="195"/>
       <c r="D16" s="1" t="s">
         <v>58</v>
       </c>
@@ -6429,7 +7261,7 @@
     </row>
     <row r="17" spans="2:26">
       <c r="B17" s="181"/>
-      <c r="C17" s="190"/>
+      <c r="C17" s="195"/>
       <c r="D17" s="1" t="s">
         <v>62</v>
       </c>
@@ -6487,7 +7319,7 @@
     </row>
     <row r="18" spans="2:26" ht="14.5" thickBot="1">
       <c r="B18" s="182"/>
-      <c r="C18" s="191"/>
+      <c r="C18" s="196"/>
       <c r="D18" s="20" t="s">
         <v>65</v>
       </c>
@@ -6547,7 +7379,7 @@
       <c r="B19" s="180" t="s">
         <v>68</v>
       </c>
-      <c r="C19" s="192" t="s">
+      <c r="C19" s="191" t="s">
         <v>69</v>
       </c>
       <c r="D19" s="5" t="s">
@@ -6607,7 +7439,7 @@
     </row>
     <row r="20" spans="2:26" ht="15" thickBot="1">
       <c r="B20" s="181"/>
-      <c r="C20" s="193"/>
+      <c r="C20" s="192"/>
       <c r="D20" s="1" t="s">
         <v>72</v>
       </c>
@@ -6665,7 +7497,7 @@
     </row>
     <row r="21" spans="2:26" ht="15" thickBot="1">
       <c r="B21" s="181"/>
-      <c r="C21" s="193"/>
+      <c r="C21" s="192"/>
       <c r="D21" s="1" t="s">
         <v>75</v>
       </c>
@@ -6723,7 +7555,7 @@
     </row>
     <row r="22" spans="2:26" ht="15" thickBot="1">
       <c r="B22" s="182"/>
-      <c r="C22" s="193"/>
+      <c r="C22" s="192"/>
       <c r="D22" s="2" t="s">
         <v>78</v>
       </c>
@@ -6783,7 +7615,7 @@
       <c r="B23" s="180" t="s">
         <v>81</v>
       </c>
-      <c r="C23" s="194" t="s">
+      <c r="C23" s="197" t="s">
         <v>82</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -6837,7 +7669,7 @@
     </row>
     <row r="24" spans="2:26">
       <c r="B24" s="181"/>
-      <c r="C24" s="193"/>
+      <c r="C24" s="192"/>
       <c r="D24" s="1" t="s">
         <v>86</v>
       </c>
@@ -6889,7 +7721,7 @@
     </row>
     <row r="25" spans="2:26">
       <c r="B25" s="181"/>
-      <c r="C25" s="193"/>
+      <c r="C25" s="192"/>
       <c r="D25" s="1" t="s">
         <v>89</v>
       </c>
@@ -6941,7 +7773,7 @@
     </row>
     <row r="26" spans="2:26" ht="14.5" thickBot="1">
       <c r="B26" s="182"/>
-      <c r="C26" s="195"/>
+      <c r="C26" s="198"/>
       <c r="D26" s="1" t="s">
         <v>93</v>
       </c>
@@ -7052,18 +7884,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B15:B18"/>
+    <mergeCell ref="C15:C18"/>
+    <mergeCell ref="B19:B22"/>
+    <mergeCell ref="C19:C22"/>
+    <mergeCell ref="B23:B26"/>
+    <mergeCell ref="C23:C26"/>
     <mergeCell ref="B3:B6"/>
     <mergeCell ref="C3:C6"/>
     <mergeCell ref="B7:B10"/>
     <mergeCell ref="C7:C10"/>
     <mergeCell ref="B11:B14"/>
     <mergeCell ref="C11:C14"/>
-    <mergeCell ref="B15:B18"/>
-    <mergeCell ref="C15:C18"/>
-    <mergeCell ref="B19:B22"/>
-    <mergeCell ref="C19:C22"/>
-    <mergeCell ref="B23:B26"/>
-    <mergeCell ref="C23:C26"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7126,10 +7958,10 @@
       </c>
     </row>
     <row r="3" spans="2:15">
-      <c r="B3" s="199" t="s">
+      <c r="B3" s="200" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="199" t="s">
+      <c r="C3" s="200" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -7170,8 +8002,8 @@
       </c>
     </row>
     <row r="4" spans="2:15">
-      <c r="B4" s="199"/>
-      <c r="C4" s="199"/>
+      <c r="B4" s="200"/>
+      <c r="C4" s="200"/>
       <c r="D4" s="1" t="s">
         <v>12</v>
       </c>
@@ -7210,8 +8042,8 @@
       </c>
     </row>
     <row r="5" spans="2:15">
-      <c r="B5" s="199"/>
-      <c r="C5" s="199"/>
+      <c r="B5" s="200"/>
+      <c r="C5" s="200"/>
       <c r="D5" s="1" t="s">
         <v>15</v>
       </c>
@@ -7250,8 +8082,8 @@
       </c>
     </row>
     <row r="6" spans="2:15">
-      <c r="B6" s="199"/>
-      <c r="C6" s="199"/>
+      <c r="B6" s="200"/>
+      <c r="C6" s="200"/>
       <c r="D6" s="1" t="s">
         <v>15</v>
       </c>
@@ -7290,10 +8122,10 @@
       </c>
     </row>
     <row r="7" spans="2:15">
-      <c r="B7" s="200" t="s">
+      <c r="B7" s="199" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="200" t="s">
+      <c r="C7" s="199" t="s">
         <v>21</v>
       </c>
       <c r="D7" s="1" t="s">
@@ -7334,8 +8166,8 @@
       </c>
     </row>
     <row r="8" spans="2:15">
-      <c r="B8" s="200"/>
-      <c r="C8" s="200"/>
+      <c r="B8" s="199"/>
+      <c r="C8" s="199"/>
       <c r="D8" s="1" t="s">
         <v>26</v>
       </c>
@@ -7374,8 +8206,8 @@
       </c>
     </row>
     <row r="9" spans="2:15">
-      <c r="B9" s="200"/>
-      <c r="C9" s="200"/>
+      <c r="B9" s="199"/>
+      <c r="C9" s="199"/>
       <c r="D9" s="1" t="s">
         <v>30</v>
       </c>
@@ -7414,8 +8246,8 @@
       </c>
     </row>
     <row r="10" spans="2:15">
-      <c r="B10" s="200"/>
-      <c r="C10" s="200"/>
+      <c r="B10" s="199"/>
+      <c r="C10" s="199"/>
       <c r="D10" s="1" t="s">
         <v>34</v>
       </c>
@@ -7454,10 +8286,10 @@
       </c>
     </row>
     <row r="11" spans="2:15">
-      <c r="B11" s="200" t="s">
+      <c r="B11" s="199" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="200" t="s">
+      <c r="C11" s="199" t="s">
         <v>39</v>
       </c>
       <c r="D11" s="1" t="s">
@@ -7498,8 +8330,8 @@
       </c>
     </row>
     <row r="12" spans="2:15">
-      <c r="B12" s="200"/>
-      <c r="C12" s="200"/>
+      <c r="B12" s="199"/>
+      <c r="C12" s="199"/>
       <c r="D12" s="1" t="s">
         <v>22</v>
       </c>
@@ -7538,8 +8370,8 @@
       </c>
     </row>
     <row r="13" spans="2:15">
-      <c r="B13" s="200"/>
-      <c r="C13" s="200"/>
+      <c r="B13" s="199"/>
+      <c r="C13" s="199"/>
       <c r="D13" s="1" t="s">
         <v>47</v>
       </c>
@@ -7578,8 +8410,8 @@
       </c>
     </row>
     <row r="14" spans="2:15">
-      <c r="B14" s="200"/>
-      <c r="C14" s="200"/>
+      <c r="B14" s="199"/>
+      <c r="C14" s="199"/>
       <c r="D14" s="1" t="s">
         <v>50</v>
       </c>
@@ -7618,10 +8450,10 @@
       </c>
     </row>
     <row r="15" spans="2:15">
-      <c r="B15" s="200" t="s">
+      <c r="B15" s="199" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="200" t="s">
+      <c r="C15" s="199" t="s">
         <v>53</v>
       </c>
       <c r="D15" s="1" t="s">
@@ -7662,8 +8494,8 @@
       </c>
     </row>
     <row r="16" spans="2:15">
-      <c r="B16" s="200"/>
-      <c r="C16" s="200"/>
+      <c r="B16" s="199"/>
+      <c r="C16" s="199"/>
       <c r="D16" s="1" t="s">
         <v>163</v>
       </c>
@@ -7702,8 +8534,8 @@
       </c>
     </row>
     <row r="17" spans="2:15">
-      <c r="B17" s="200"/>
-      <c r="C17" s="200"/>
+      <c r="B17" s="199"/>
+      <c r="C17" s="199"/>
       <c r="D17" s="1" t="s">
         <v>62</v>
       </c>
@@ -7742,8 +8574,8 @@
       </c>
     </row>
     <row r="18" spans="2:15">
-      <c r="B18" s="200"/>
-      <c r="C18" s="200"/>
+      <c r="B18" s="199"/>
+      <c r="C18" s="199"/>
       <c r="D18" s="105" t="s">
         <v>65</v>
       </c>
@@ -7782,10 +8614,10 @@
       </c>
     </row>
     <row r="19" spans="2:15" ht="14.5">
-      <c r="B19" s="200" t="s">
+      <c r="B19" s="199" t="s">
         <v>68</v>
       </c>
-      <c r="C19" s="200" t="s">
+      <c r="C19" s="199" t="s">
         <v>69</v>
       </c>
       <c r="D19" s="1" t="s">
@@ -7826,8 +8658,8 @@
       </c>
     </row>
     <row r="20" spans="2:15" ht="14.5">
-      <c r="B20" s="200"/>
-      <c r="C20" s="200"/>
+      <c r="B20" s="199"/>
+      <c r="C20" s="199"/>
       <c r="D20" s="1" t="s">
         <v>72</v>
       </c>
@@ -7866,8 +8698,8 @@
       </c>
     </row>
     <row r="21" spans="2:15" ht="14.5">
-      <c r="B21" s="200"/>
-      <c r="C21" s="200"/>
+      <c r="B21" s="199"/>
+      <c r="C21" s="199"/>
       <c r="D21" s="1" t="s">
         <v>75</v>
       </c>
@@ -7906,8 +8738,8 @@
       </c>
     </row>
     <row r="22" spans="2:15" ht="14.5">
-      <c r="B22" s="200"/>
-      <c r="C22" s="200"/>
+      <c r="B22" s="199"/>
+      <c r="C22" s="199"/>
       <c r="D22" s="1" t="s">
         <v>78</v>
       </c>
@@ -7946,10 +8778,10 @@
       </c>
     </row>
     <row r="23" spans="2:15">
-      <c r="B23" s="200" t="s">
+      <c r="B23" s="199" t="s">
         <v>81</v>
       </c>
-      <c r="C23" s="200" t="s">
+      <c r="C23" s="199" t="s">
         <v>82</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -7990,8 +8822,8 @@
       </c>
     </row>
     <row r="24" spans="2:15">
-      <c r="B24" s="200"/>
-      <c r="C24" s="200"/>
+      <c r="B24" s="199"/>
+      <c r="C24" s="199"/>
       <c r="D24" s="1" t="s">
         <v>86</v>
       </c>
@@ -8030,8 +8862,8 @@
       </c>
     </row>
     <row r="25" spans="2:15">
-      <c r="B25" s="200"/>
-      <c r="C25" s="200"/>
+      <c r="B25" s="199"/>
+      <c r="C25" s="199"/>
       <c r="D25" s="1" t="s">
         <v>89</v>
       </c>
@@ -8070,8 +8902,8 @@
       </c>
     </row>
     <row r="26" spans="2:15">
-      <c r="B26" s="200"/>
-      <c r="C26" s="200"/>
+      <c r="B26" s="199"/>
+      <c r="C26" s="199"/>
       <c r="D26" s="1" t="s">
         <v>93</v>
       </c>
@@ -8148,18 +8980,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="C7:C10"/>
+    <mergeCell ref="B11:B14"/>
+    <mergeCell ref="C11:C14"/>
     <mergeCell ref="B15:B18"/>
     <mergeCell ref="C15:C18"/>
     <mergeCell ref="B19:B22"/>
     <mergeCell ref="C19:C22"/>
     <mergeCell ref="B23:B26"/>
     <mergeCell ref="C23:C26"/>
-    <mergeCell ref="B3:B6"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="C7:C10"/>
-    <mergeCell ref="B11:B14"/>
-    <mergeCell ref="C11:C14"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8214,7 +9046,7 @@
       <c r="A2" s="186" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="196" t="s">
+      <c r="B2" s="189" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="5" t="s">
@@ -8251,7 +9083,7 @@
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="187"/>
-      <c r="B3" s="196"/>
+      <c r="B3" s="189"/>
       <c r="C3" s="1" t="s">
         <v>12</v>
       </c>
@@ -8286,7 +9118,7 @@
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="187"/>
-      <c r="B4" s="196"/>
+      <c r="B4" s="189"/>
       <c r="C4" s="1" t="s">
         <v>15</v>
       </c>
@@ -8321,7 +9153,7 @@
     </row>
     <row r="5" spans="1:13" ht="14.5" thickBot="1">
       <c r="A5" s="188"/>
-      <c r="B5" s="197"/>
+      <c r="B5" s="190"/>
       <c r="C5" s="11" t="s">
         <v>15</v>
       </c>
@@ -8358,7 +9190,7 @@
       <c r="A6" s="180" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="192" t="s">
+      <c r="B6" s="191" t="s">
         <v>21</v>
       </c>
       <c r="C6" s="5" t="s">
@@ -8395,7 +9227,7 @@
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="181"/>
-      <c r="B7" s="193"/>
+      <c r="B7" s="192"/>
       <c r="C7" s="1" t="s">
         <v>26</v>
       </c>
@@ -8430,7 +9262,7 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="181"/>
-      <c r="B8" s="193"/>
+      <c r="B8" s="192"/>
       <c r="C8" s="1" t="s">
         <v>30</v>
       </c>
@@ -8465,7 +9297,7 @@
     </row>
     <row r="9" spans="1:13" ht="14.5" thickBot="1">
       <c r="A9" s="182"/>
-      <c r="B9" s="198"/>
+      <c r="B9" s="193"/>
       <c r="C9" s="11" t="s">
         <v>34</v>
       </c>
@@ -8502,7 +9334,7 @@
       <c r="A10" s="180" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="192" t="s">
+      <c r="B10" s="191" t="s">
         <v>39</v>
       </c>
       <c r="C10" s="5" t="s">
@@ -8539,7 +9371,7 @@
     </row>
     <row r="11" spans="1:13">
       <c r="A11" s="181"/>
-      <c r="B11" s="193"/>
+      <c r="B11" s="192"/>
       <c r="C11" s="1" t="s">
         <v>22</v>
       </c>
@@ -8574,7 +9406,7 @@
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="181"/>
-      <c r="B12" s="193"/>
+      <c r="B12" s="192"/>
       <c r="C12" s="1" t="s">
         <v>47</v>
       </c>
@@ -8609,7 +9441,7 @@
     </row>
     <row r="13" spans="1:13" ht="14.5" thickBot="1">
       <c r="A13" s="182"/>
-      <c r="B13" s="198"/>
+      <c r="B13" s="193"/>
       <c r="C13" s="11" t="s">
         <v>50</v>
       </c>
@@ -8646,7 +9478,7 @@
       <c r="A14" s="180" t="s">
         <v>52</v>
       </c>
-      <c r="B14" s="189" t="s">
+      <c r="B14" s="194" t="s">
         <v>53</v>
       </c>
       <c r="C14" s="5" t="s">
@@ -8683,7 +9515,7 @@
     </row>
     <row r="15" spans="1:13">
       <c r="A15" s="181"/>
-      <c r="B15" s="190"/>
+      <c r="B15" s="195"/>
       <c r="C15" s="1" t="s">
         <v>58</v>
       </c>
@@ -8718,7 +9550,7 @@
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="181"/>
-      <c r="B16" s="190"/>
+      <c r="B16" s="195"/>
       <c r="C16" s="1" t="s">
         <v>62</v>
       </c>
@@ -8753,7 +9585,7 @@
     </row>
     <row r="17" spans="1:12" ht="14.5" thickBot="1">
       <c r="A17" s="182"/>
-      <c r="B17" s="191"/>
+      <c r="B17" s="196"/>
       <c r="C17" s="20" t="s">
         <v>65</v>
       </c>
@@ -8790,7 +9622,7 @@
       <c r="A18" s="180" t="s">
         <v>68</v>
       </c>
-      <c r="B18" s="192" t="s">
+      <c r="B18" s="191" t="s">
         <v>69</v>
       </c>
       <c r="C18" s="5" t="s">
@@ -8827,7 +9659,7 @@
     </row>
     <row r="19" spans="1:12">
       <c r="A19" s="181"/>
-      <c r="B19" s="193"/>
+      <c r="B19" s="192"/>
       <c r="C19" s="1" t="s">
         <v>72</v>
       </c>
@@ -8862,7 +9694,7 @@
     </row>
     <row r="20" spans="1:12">
       <c r="A20" s="181"/>
-      <c r="B20" s="193"/>
+      <c r="B20" s="192"/>
       <c r="C20" s="1" t="s">
         <v>75</v>
       </c>
@@ -8897,7 +9729,7 @@
     </row>
     <row r="21" spans="1:12" ht="14.5" thickBot="1">
       <c r="A21" s="182"/>
-      <c r="B21" s="193"/>
+      <c r="B21" s="192"/>
       <c r="C21" s="2" t="s">
         <v>78</v>
       </c>
@@ -8934,7 +9766,7 @@
       <c r="A22" s="180" t="s">
         <v>81</v>
       </c>
-      <c r="B22" s="194" t="s">
+      <c r="B22" s="197" t="s">
         <v>82</v>
       </c>
       <c r="C22" s="1" t="s">
@@ -8971,7 +9803,7 @@
     </row>
     <row r="23" spans="1:12">
       <c r="A23" s="181"/>
-      <c r="B23" s="193"/>
+      <c r="B23" s="192"/>
       <c r="C23" s="1" t="s">
         <v>86</v>
       </c>
@@ -9006,7 +9838,7 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24" s="181"/>
-      <c r="B24" s="193"/>
+      <c r="B24" s="192"/>
       <c r="C24" s="1" t="s">
         <v>89</v>
       </c>
@@ -9041,7 +9873,7 @@
     </row>
     <row r="25" spans="1:12" ht="14.5" thickBot="1">
       <c r="A25" s="182"/>
-      <c r="B25" s="195"/>
+      <c r="B25" s="198"/>
       <c r="C25" s="1" t="s">
         <v>93</v>
       </c>
@@ -9114,18 +9946,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="B10:B13"/>
     <mergeCell ref="A14:A17"/>
     <mergeCell ref="B14:B17"/>
     <mergeCell ref="A18:A21"/>
     <mergeCell ref="B18:B21"/>
     <mergeCell ref="A22:A25"/>
     <mergeCell ref="B22:B25"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="B10:B13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9531,21 +10363,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="56">
-      <c r="G1" s="208" t="s">
+      <c r="G1" s="201" t="s">
         <v>105</v>
       </c>
-      <c r="H1" s="208"/>
-      <c r="I1" s="208"/>
-      <c r="J1" s="208"/>
-      <c r="K1" s="208"/>
+      <c r="H1" s="201"/>
+      <c r="I1" s="201"/>
+      <c r="J1" s="201"/>
+      <c r="K1" s="201"/>
       <c r="L1" s="80"/>
-      <c r="M1" s="208" t="s">
+      <c r="M1" s="201" t="s">
         <v>106</v>
       </c>
-      <c r="N1" s="208"/>
-      <c r="O1" s="208"/>
-      <c r="P1" s="208"/>
-      <c r="Q1" s="208"/>
+      <c r="N1" s="201"/>
+      <c r="O1" s="201"/>
+      <c r="P1" s="201"/>
+      <c r="Q1" s="201"/>
       <c r="R1" s="81"/>
       <c r="S1" s="82" t="s">
         <v>107</v>
@@ -9617,7 +10449,7 @@
       <c r="A3" s="186" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="209" t="s">
+      <c r="B3" s="202" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="5" t="s">
@@ -9678,7 +10510,7 @@
     </row>
     <row r="4" spans="1:22">
       <c r="A4" s="187"/>
-      <c r="B4" s="209"/>
+      <c r="B4" s="202"/>
       <c r="C4" s="1" t="s">
         <v>12</v>
       </c>
@@ -9737,7 +10569,7 @@
     </row>
     <row r="5" spans="1:22">
       <c r="A5" s="187"/>
-      <c r="B5" s="209"/>
+      <c r="B5" s="202"/>
       <c r="C5" s="1" t="s">
         <v>15</v>
       </c>
@@ -9796,7 +10628,7 @@
     </row>
     <row r="6" spans="1:22" ht="14.5" thickBot="1">
       <c r="A6" s="188"/>
-      <c r="B6" s="210"/>
+      <c r="B6" s="203"/>
       <c r="C6" s="11" t="s">
         <v>15</v>
       </c>
@@ -9899,7 +10731,7 @@
       <c r="A8" s="180" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="203" t="s">
+      <c r="B8" s="204" t="s">
         <v>21</v>
       </c>
       <c r="C8" s="5" t="s">
@@ -9960,7 +10792,7 @@
     </row>
     <row r="9" spans="1:22">
       <c r="A9" s="181"/>
-      <c r="B9" s="202"/>
+      <c r="B9" s="205"/>
       <c r="C9" s="1" t="s">
         <v>26</v>
       </c>
@@ -10019,7 +10851,7 @@
     </row>
     <row r="10" spans="1:22">
       <c r="A10" s="181"/>
-      <c r="B10" s="202"/>
+      <c r="B10" s="205"/>
       <c r="C10" s="1" t="s">
         <v>30</v>
       </c>
@@ -10078,7 +10910,7 @@
     </row>
     <row r="11" spans="1:22" ht="14.5" thickBot="1">
       <c r="A11" s="182"/>
-      <c r="B11" s="204"/>
+      <c r="B11" s="206"/>
       <c r="C11" s="11" t="s">
         <v>34</v>
       </c>
@@ -10181,7 +11013,7 @@
       <c r="A13" s="180" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="203" t="s">
+      <c r="B13" s="204" t="s">
         <v>39</v>
       </c>
       <c r="C13" s="5" t="s">
@@ -10242,7 +11074,7 @@
     </row>
     <row r="14" spans="1:22">
       <c r="A14" s="181"/>
-      <c r="B14" s="202"/>
+      <c r="B14" s="205"/>
       <c r="C14" s="1" t="s">
         <v>22</v>
       </c>
@@ -10301,7 +11133,7 @@
     </row>
     <row r="15" spans="1:22">
       <c r="A15" s="181"/>
-      <c r="B15" s="202"/>
+      <c r="B15" s="205"/>
       <c r="C15" s="1" t="s">
         <v>47</v>
       </c>
@@ -10360,7 +11192,7 @@
     </row>
     <row r="16" spans="1:22" ht="14.5" thickBot="1">
       <c r="A16" s="182"/>
-      <c r="B16" s="204"/>
+      <c r="B16" s="206"/>
       <c r="C16" s="11" t="s">
         <v>50</v>
       </c>
@@ -10463,7 +11295,7 @@
       <c r="A18" s="180" t="s">
         <v>52</v>
       </c>
-      <c r="B18" s="205" t="s">
+      <c r="B18" s="208" t="s">
         <v>53</v>
       </c>
       <c r="C18" s="5" t="s">
@@ -10524,7 +11356,7 @@
     </row>
     <row r="19" spans="1:22">
       <c r="A19" s="181"/>
-      <c r="B19" s="206"/>
+      <c r="B19" s="209"/>
       <c r="C19" s="1" t="s">
         <v>58</v>
       </c>
@@ -10583,7 +11415,7 @@
     </row>
     <row r="20" spans="1:22">
       <c r="A20" s="181"/>
-      <c r="B20" s="206"/>
+      <c r="B20" s="209"/>
       <c r="C20" s="1" t="s">
         <v>62</v>
       </c>
@@ -10642,7 +11474,7 @@
     </row>
     <row r="21" spans="1:22" ht="14.5" thickBot="1">
       <c r="A21" s="182"/>
-      <c r="B21" s="207"/>
+      <c r="B21" s="210"/>
       <c r="C21" s="20" t="s">
         <v>65</v>
       </c>
@@ -10745,7 +11577,7 @@
       <c r="A23" s="180" t="s">
         <v>68</v>
       </c>
-      <c r="B23" s="203" t="s">
+      <c r="B23" s="204" t="s">
         <v>69</v>
       </c>
       <c r="C23" s="5" t="s">
@@ -10806,7 +11638,7 @@
     </row>
     <row r="24" spans="1:22" ht="15" thickBot="1">
       <c r="A24" s="181"/>
-      <c r="B24" s="202"/>
+      <c r="B24" s="205"/>
       <c r="C24" s="1" t="s">
         <v>72</v>
       </c>
@@ -10865,7 +11697,7 @@
     </row>
     <row r="25" spans="1:22" ht="15" thickBot="1">
       <c r="A25" s="181"/>
-      <c r="B25" s="202"/>
+      <c r="B25" s="205"/>
       <c r="C25" s="1" t="s">
         <v>75</v>
       </c>
@@ -10924,7 +11756,7 @@
     </row>
     <row r="26" spans="1:22" ht="15" thickBot="1">
       <c r="A26" s="182"/>
-      <c r="B26" s="202"/>
+      <c r="B26" s="205"/>
       <c r="C26" s="2" t="s">
         <v>78</v>
       </c>
@@ -11027,7 +11859,7 @@
       <c r="A28" s="180" t="s">
         <v>81</v>
       </c>
-      <c r="B28" s="201" t="s">
+      <c r="B28" s="207" t="s">
         <v>82</v>
       </c>
       <c r="C28" s="1" t="s">
@@ -11084,7 +11916,7 @@
     </row>
     <row r="29" spans="1:22">
       <c r="A29" s="181"/>
-      <c r="B29" s="202"/>
+      <c r="B29" s="205"/>
       <c r="C29" s="1" t="s">
         <v>86</v>
       </c>
@@ -11139,7 +11971,7 @@
     </row>
     <row r="30" spans="1:22">
       <c r="A30" s="181"/>
-      <c r="B30" s="202"/>
+      <c r="B30" s="205"/>
       <c r="C30" s="1" t="s">
         <v>89</v>
       </c>
@@ -11194,7 +12026,7 @@
     </row>
     <row r="31" spans="1:22">
       <c r="A31" s="181"/>
-      <c r="B31" s="202"/>
+      <c r="B31" s="205"/>
       <c r="C31" s="2" t="s">
         <v>93</v>
       </c>
@@ -11325,12 +12157,6 @@
     <filterColumn colId="15" showButton="0"/>
   </autoFilter>
   <mergeCells count="14">
-    <mergeCell ref="G1:K1"/>
-    <mergeCell ref="M1:Q1"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="B3:B6"/>
-    <mergeCell ref="A8:A11"/>
-    <mergeCell ref="B8:B11"/>
     <mergeCell ref="A28:A31"/>
     <mergeCell ref="B28:B31"/>
     <mergeCell ref="A13:A16"/>
@@ -11339,6 +12165,12 @@
     <mergeCell ref="B18:B21"/>
     <mergeCell ref="A23:A26"/>
     <mergeCell ref="B23:B26"/>
+    <mergeCell ref="G1:K1"/>
+    <mergeCell ref="M1:Q1"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="B8:B11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11494,10 +12326,10 @@
       </c>
     </row>
     <row r="3" spans="1:31">
-      <c r="A3" s="199" t="s">
+      <c r="A3" s="200" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="199" t="s">
+      <c r="B3" s="200" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -11584,8 +12416,8 @@
       <c r="AE3" s="26"/>
     </row>
     <row r="4" spans="1:31">
-      <c r="A4" s="199"/>
-      <c r="B4" s="199"/>
+      <c r="A4" s="200"/>
+      <c r="B4" s="200"/>
       <c r="C4" s="1" t="s">
         <v>12</v>
       </c>
@@ -11669,8 +12501,8 @@
       <c r="AE4" s="26"/>
     </row>
     <row r="5" spans="1:31">
-      <c r="A5" s="199"/>
-      <c r="B5" s="199"/>
+      <c r="A5" s="200"/>
+      <c r="B5" s="200"/>
       <c r="C5" s="1" t="s">
         <v>15</v>
       </c>
@@ -11755,8 +12587,8 @@
       <c r="AE5" s="26"/>
     </row>
     <row r="6" spans="1:31">
-      <c r="A6" s="199"/>
-      <c r="B6" s="199"/>
+      <c r="A6" s="200"/>
+      <c r="B6" s="200"/>
       <c r="C6" s="1" t="s">
         <v>15</v>
       </c>
@@ -11892,10 +12724,10 @@
       </c>
     </row>
     <row r="8" spans="1:31">
-      <c r="A8" s="200" t="s">
+      <c r="A8" s="199" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="200" t="s">
+      <c r="B8" s="199" t="s">
         <v>21</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -11982,8 +12814,8 @@
       <c r="AE8" s="26"/>
     </row>
     <row r="9" spans="1:31">
-      <c r="A9" s="200"/>
-      <c r="B9" s="200"/>
+      <c r="A9" s="199"/>
+      <c r="B9" s="199"/>
       <c r="C9" s="1" t="s">
         <v>26</v>
       </c>
@@ -12068,8 +12900,8 @@
       <c r="AE9" s="26"/>
     </row>
     <row r="10" spans="1:31">
-      <c r="A10" s="200"/>
-      <c r="B10" s="200"/>
+      <c r="A10" s="199"/>
+      <c r="B10" s="199"/>
       <c r="C10" s="1" t="s">
         <v>30</v>
       </c>
@@ -12154,8 +12986,8 @@
       <c r="AE10" s="26"/>
     </row>
     <row r="11" spans="1:31">
-      <c r="A11" s="200"/>
-      <c r="B11" s="200"/>
+      <c r="A11" s="199"/>
+      <c r="B11" s="199"/>
       <c r="C11" s="1" t="s">
         <v>34</v>
       </c>
@@ -12291,10 +13123,10 @@
       </c>
     </row>
     <row r="13" spans="1:31">
-      <c r="A13" s="200" t="s">
+      <c r="A13" s="199" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="200" t="s">
+      <c r="B13" s="199" t="s">
         <v>39</v>
       </c>
       <c r="C13" s="1" t="s">
@@ -12381,8 +13213,8 @@
       <c r="AE13" s="26"/>
     </row>
     <row r="14" spans="1:31">
-      <c r="A14" s="200"/>
-      <c r="B14" s="200"/>
+      <c r="A14" s="199"/>
+      <c r="B14" s="199"/>
       <c r="C14" s="1" t="s">
         <v>22</v>
       </c>
@@ -12466,8 +13298,8 @@
       <c r="AE14" s="26"/>
     </row>
     <row r="15" spans="1:31">
-      <c r="A15" s="200"/>
-      <c r="B15" s="200"/>
+      <c r="A15" s="199"/>
+      <c r="B15" s="199"/>
       <c r="C15" s="1" t="s">
         <v>47</v>
       </c>
@@ -12552,8 +13384,8 @@
       <c r="AE15" s="26"/>
     </row>
     <row r="16" spans="1:31">
-      <c r="A16" s="200"/>
-      <c r="B16" s="200"/>
+      <c r="A16" s="199"/>
+      <c r="B16" s="199"/>
       <c r="C16" s="1" t="s">
         <v>50</v>
       </c>
@@ -12688,10 +13520,10 @@
       </c>
     </row>
     <row r="18" spans="1:31">
-      <c r="A18" s="200" t="s">
+      <c r="A18" s="199" t="s">
         <v>52</v>
       </c>
-      <c r="B18" s="200" t="s">
+      <c r="B18" s="199" t="s">
         <v>53</v>
       </c>
       <c r="C18" s="1" t="s">
@@ -12777,8 +13609,8 @@
       <c r="AE18" s="26"/>
     </row>
     <row r="19" spans="1:31">
-      <c r="A19" s="200"/>
-      <c r="B19" s="200"/>
+      <c r="A19" s="199"/>
+      <c r="B19" s="199"/>
       <c r="C19" s="1" t="s">
         <v>58</v>
       </c>
@@ -12862,8 +13694,8 @@
       <c r="AE19" s="26"/>
     </row>
     <row r="20" spans="1:31">
-      <c r="A20" s="200"/>
-      <c r="B20" s="200"/>
+      <c r="A20" s="199"/>
+      <c r="B20" s="199"/>
       <c r="C20" s="1" t="s">
         <v>62</v>
       </c>
@@ -12947,8 +13779,8 @@
       <c r="AE20" s="26"/>
     </row>
     <row r="21" spans="1:31">
-      <c r="A21" s="200"/>
-      <c r="B21" s="200"/>
+      <c r="A21" s="199"/>
+      <c r="B21" s="199"/>
       <c r="C21" s="105" t="s">
         <v>65</v>
       </c>
@@ -13084,10 +13916,10 @@
       </c>
     </row>
     <row r="23" spans="1:31" ht="14.5">
-      <c r="A23" s="200" t="s">
+      <c r="A23" s="199" t="s">
         <v>68</v>
       </c>
-      <c r="B23" s="200" t="s">
+      <c r="B23" s="199" t="s">
         <v>69</v>
       </c>
       <c r="C23" s="1" t="s">
@@ -13174,8 +14006,8 @@
       <c r="AE23" s="26"/>
     </row>
     <row r="24" spans="1:31" ht="14.5">
-      <c r="A24" s="200"/>
-      <c r="B24" s="200"/>
+      <c r="A24" s="199"/>
+      <c r="B24" s="199"/>
       <c r="C24" s="1" t="s">
         <v>72</v>
       </c>
@@ -13259,8 +14091,8 @@
       <c r="AE24" s="26"/>
     </row>
     <row r="25" spans="1:31" ht="14.5">
-      <c r="A25" s="200"/>
-      <c r="B25" s="200"/>
+      <c r="A25" s="199"/>
+      <c r="B25" s="199"/>
       <c r="C25" s="1" t="s">
         <v>75</v>
       </c>
@@ -13345,8 +14177,8 @@
       <c r="AE25" s="26"/>
     </row>
     <row r="26" spans="1:31" ht="16" customHeight="1">
-      <c r="A26" s="200"/>
-      <c r="B26" s="200"/>
+      <c r="A26" s="199"/>
+      <c r="B26" s="199"/>
       <c r="C26" s="1" t="s">
         <v>78</v>
       </c>
@@ -13481,10 +14313,10 @@
       </c>
     </row>
     <row r="28" spans="1:31">
-      <c r="A28" s="200" t="s">
+      <c r="A28" s="199" t="s">
         <v>81</v>
       </c>
-      <c r="B28" s="200" t="s">
+      <c r="B28" s="199" t="s">
         <v>82</v>
       </c>
       <c r="C28" s="1" t="s">
@@ -13563,8 +14395,8 @@
       <c r="AE28" s="26"/>
     </row>
     <row r="29" spans="1:31">
-      <c r="A29" s="200"/>
-      <c r="B29" s="200"/>
+      <c r="A29" s="199"/>
+      <c r="B29" s="199"/>
       <c r="C29" s="1" t="s">
         <v>86</v>
       </c>
@@ -13641,8 +14473,8 @@
       <c r="AE29" s="26"/>
     </row>
     <row r="30" spans="1:31">
-      <c r="A30" s="200"/>
-      <c r="B30" s="200"/>
+      <c r="A30" s="199"/>
+      <c r="B30" s="199"/>
       <c r="C30" s="1" t="s">
         <v>89</v>
       </c>
@@ -13719,8 +14551,8 @@
       <c r="AE30" s="26"/>
     </row>
     <row r="31" spans="1:31">
-      <c r="A31" s="200"/>
-      <c r="B31" s="200"/>
+      <c r="A31" s="199"/>
+      <c r="B31" s="199"/>
       <c r="C31" s="1" t="s">
         <v>93</v>
       </c>

</xml_diff>